<commit_message>
actualizaciones de cronograma y ajuste a vistas
</commit_message>
<xml_diff>
--- a/data/metas.xlsx
+++ b/data/metas.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\POI\Seguimiento_Metas\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROYECTOS - 2026 (DEV)\DEV - POI\Insights_POI\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3FB119C-9823-4D0C-9D03-3883C60A5E83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CDF2BCE-AE11-4B87-8108-4E818414E7F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$310</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$323</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1864" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1942" uniqueCount="386">
   <si>
     <t>ID_META</t>
   </si>
@@ -1152,7 +1152,46 @@
     <t>Fernando Yupanqui</t>
   </si>
   <si>
-    <t>diseñadora</t>
+    <t>M00152</t>
+  </si>
+  <si>
+    <t>M00195</t>
+  </si>
+  <si>
+    <t>M00312</t>
+  </si>
+  <si>
+    <t>M00313</t>
+  </si>
+  <si>
+    <t>M00314</t>
+  </si>
+  <si>
+    <t>M00315</t>
+  </si>
+  <si>
+    <t>M00316</t>
+  </si>
+  <si>
+    <t>M00317</t>
+  </si>
+  <si>
+    <t>M00318</t>
+  </si>
+  <si>
+    <t>M00319</t>
+  </si>
+  <si>
+    <t>M00320</t>
+  </si>
+  <si>
+    <t>M00321</t>
+  </si>
+  <si>
+    <t>M00322</t>
+  </si>
+  <si>
+    <t>Diseñadora</t>
   </si>
 </sst>
 </file>
@@ -1507,7 +1546,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J310"/>
+  <dimension ref="A1:J323"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -1516,7 +1555,7 @@
     <col min="5" max="5" width="18.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="70.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="106.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="71.42578125" style="1" customWidth="1"/>
     <col min="9" max="9" width="18.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="22.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="16384" width="9.140625" style="1"/>
@@ -6388,7 +6427,7 @@
     </row>
     <row r="153" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A153" s="1" t="s">
-        <v>160</v>
+        <v>372</v>
       </c>
       <c r="B153" s="1">
         <v>2026</v>
@@ -6420,7 +6459,7 @@
     </row>
     <row r="154" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A154" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B154" s="1">
         <v>2026</v>
@@ -6452,7 +6491,7 @@
     </row>
     <row r="155" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A155" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B155" s="1">
         <v>2026</v>
@@ -6484,7 +6523,7 @@
     </row>
     <row r="156" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A156" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B156" s="1">
         <v>2026</v>
@@ -6516,7 +6555,7 @@
     </row>
     <row r="157" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A157" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B157" s="1">
         <v>2026</v>
@@ -6548,7 +6587,7 @@
     </row>
     <row r="158" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A158" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B158" s="1">
         <v>2026</v>
@@ -6580,7 +6619,7 @@
     </row>
     <row r="159" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A159" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B159" s="1">
         <v>2026</v>
@@ -6612,7 +6651,7 @@
     </row>
     <row r="160" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A160" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B160" s="1">
         <v>2026</v>
@@ -6644,7 +6683,7 @@
     </row>
     <row r="161" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A161" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B161" s="1">
         <v>2026</v>
@@ -6676,7 +6715,7 @@
     </row>
     <row r="162" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A162" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B162" s="1">
         <v>2026</v>
@@ -6708,7 +6747,7 @@
     </row>
     <row r="163" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A163" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B163" s="1">
         <v>2026</v>
@@ -6740,7 +6779,7 @@
     </row>
     <row r="164" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A164" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B164" s="1">
         <v>2026</v>
@@ -6772,7 +6811,7 @@
     </row>
     <row r="165" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A165" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B165" s="1">
         <v>2026</v>
@@ -6804,7 +6843,7 @@
     </row>
     <row r="166" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A166" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B166" s="1">
         <v>2026</v>
@@ -6836,7 +6875,7 @@
     </row>
     <row r="167" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A167" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B167" s="1">
         <v>2026</v>
@@ -6868,7 +6907,7 @@
     </row>
     <row r="168" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A168" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B168" s="1">
         <v>2026</v>
@@ -6900,7 +6939,7 @@
     </row>
     <row r="169" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A169" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B169" s="1">
         <v>2026</v>
@@ -6932,7 +6971,7 @@
     </row>
     <row r="170" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A170" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B170" s="1">
         <v>2026</v>
@@ -6964,7 +7003,7 @@
     </row>
     <row r="171" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A171" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B171" s="1">
         <v>2026</v>
@@ -6996,7 +7035,7 @@
     </row>
     <row r="172" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A172" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B172" s="1">
         <v>2026</v>
@@ -7028,7 +7067,7 @@
     </row>
     <row r="173" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A173" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B173" s="1">
         <v>2026</v>
@@ -7060,7 +7099,7 @@
     </row>
     <row r="174" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A174" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B174" s="1">
         <v>2026</v>
@@ -7092,7 +7131,7 @@
     </row>
     <row r="175" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A175" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B175" s="1">
         <v>2026</v>
@@ -7124,7 +7163,7 @@
     </row>
     <row r="176" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A176" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B176" s="1">
         <v>2026</v>
@@ -7156,7 +7195,7 @@
     </row>
     <row r="177" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A177" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B177" s="1">
         <v>2026</v>
@@ -7188,7 +7227,7 @@
     </row>
     <row r="178" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A178" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B178" s="1">
         <v>2026</v>
@@ -7220,7 +7259,7 @@
     </row>
     <row r="179" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A179" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B179" s="1">
         <v>2026</v>
@@ -7252,7 +7291,7 @@
     </row>
     <row r="180" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A180" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B180" s="1">
         <v>2026</v>
@@ -7284,7 +7323,7 @@
     </row>
     <row r="181" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A181" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B181" s="1">
         <v>2026</v>
@@ -7316,7 +7355,7 @@
     </row>
     <row r="182" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A182" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B182" s="1">
         <v>2026</v>
@@ -7348,7 +7387,7 @@
     </row>
     <row r="183" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A183" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B183" s="1">
         <v>2026</v>
@@ -7380,7 +7419,7 @@
     </row>
     <row r="184" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A184" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B184" s="1">
         <v>2026</v>
@@ -7412,7 +7451,7 @@
     </row>
     <row r="185" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A185" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B185" s="1">
         <v>2026</v>
@@ -7444,7 +7483,7 @@
     </row>
     <row r="186" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A186" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B186" s="1">
         <v>2026</v>
@@ -7476,7 +7515,7 @@
     </row>
     <row r="187" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A187" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B187" s="1">
         <v>2026</v>
@@ -7508,7 +7547,7 @@
     </row>
     <row r="188" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A188" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B188" s="1">
         <v>2026</v>
@@ -7540,7 +7579,7 @@
     </row>
     <row r="189" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A189" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B189" s="1">
         <v>2026</v>
@@ -7572,7 +7611,7 @@
     </row>
     <row r="190" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A190" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B190" s="1">
         <v>2026</v>
@@ -7604,7 +7643,7 @@
     </row>
     <row r="191" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A191" s="1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B191" s="1">
         <v>2026</v>
@@ -7636,7 +7675,7 @@
     </row>
     <row r="192" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A192" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B192" s="1">
         <v>2026</v>
@@ -7668,7 +7707,7 @@
     </row>
     <row r="193" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A193" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B193" s="1">
         <v>2026</v>
@@ -7700,7 +7739,7 @@
     </row>
     <row r="194" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A194" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B194" s="1">
         <v>2026</v>
@@ -7732,7 +7771,7 @@
     </row>
     <row r="195" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A195" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B195" s="1">
         <v>2026</v>
@@ -7764,7 +7803,7 @@
     </row>
     <row r="196" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A196" s="1" t="s">
-        <v>203</v>
+        <v>373</v>
       </c>
       <c r="B196" s="1">
         <v>2026</v>
@@ -7796,7 +7835,7 @@
     </row>
     <row r="197" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A197" s="1" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B197" s="1">
         <v>2026</v>
@@ -7828,7 +7867,7 @@
     </row>
     <row r="198" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A198" s="1" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B198" s="1">
         <v>2026</v>
@@ -7860,7 +7899,7 @@
     </row>
     <row r="199" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A199" s="1" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B199" s="1">
         <v>2026</v>
@@ -7892,7 +7931,7 @@
     </row>
     <row r="200" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A200" s="1" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B200" s="1">
         <v>2026</v>
@@ -7924,7 +7963,7 @@
     </row>
     <row r="201" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A201" s="1" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B201" s="1">
         <v>2026</v>
@@ -7956,7 +7995,7 @@
     </row>
     <row r="202" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A202" s="1" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B202" s="1">
         <v>2026</v>
@@ -7988,7 +8027,7 @@
     </row>
     <row r="203" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A203" s="1" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B203" s="1">
         <v>2026</v>
@@ -8020,7 +8059,7 @@
     </row>
     <row r="204" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A204" s="1" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B204" s="1">
         <v>2026</v>
@@ -8052,7 +8091,7 @@
     </row>
     <row r="205" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A205" s="1" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B205" s="1">
         <v>2026</v>
@@ -8084,7 +8123,7 @@
     </row>
     <row r="206" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A206" s="1" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B206" s="1">
         <v>2026</v>
@@ -8116,7 +8155,7 @@
     </row>
     <row r="207" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A207" s="1" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B207" s="1">
         <v>2026</v>
@@ -8148,7 +8187,7 @@
     </row>
     <row r="208" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A208" s="1" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B208" s="1">
         <v>2026</v>
@@ -8180,7 +8219,7 @@
     </row>
     <row r="209" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A209" s="1" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B209" s="1">
         <v>2026</v>
@@ -8212,7 +8251,7 @@
     </row>
     <row r="210" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A210" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B210" s="1">
         <v>2026</v>
@@ -8244,7 +8283,7 @@
     </row>
     <row r="211" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A211" s="1" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B211" s="1">
         <v>2026</v>
@@ -8276,7 +8315,7 @@
     </row>
     <row r="212" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A212" s="1" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B212" s="1">
         <v>2026</v>
@@ -8308,7 +8347,7 @@
     </row>
     <row r="213" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A213" s="1" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B213" s="1">
         <v>2026</v>
@@ -8340,7 +8379,7 @@
     </row>
     <row r="214" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A214" s="1" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B214" s="1">
         <v>2026</v>
@@ -8372,7 +8411,7 @@
     </row>
     <row r="215" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A215" s="1" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B215" s="1">
         <v>2026</v>
@@ -8404,7 +8443,7 @@
     </row>
     <row r="216" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A216" s="1" t="s">
-        <v>266</v>
+        <v>221</v>
       </c>
       <c r="B216" s="1">
         <v>2026</v>
@@ -8436,19 +8475,19 @@
     </row>
     <row r="217" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A217" s="1" t="s">
-        <v>267</v>
+        <v>222</v>
       </c>
       <c r="B217" s="1">
         <v>2026</v>
       </c>
       <c r="C217" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D217" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E217" s="1" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="F217" s="1" t="s">
         <v>361</v>
@@ -8460,7 +8499,7 @@
         <v>238</v>
       </c>
       <c r="I217" s="1">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J217" s="1">
         <v>0</v>
@@ -8468,19 +8507,19 @@
     </row>
     <row r="218" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A218" s="1" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B218" s="1">
         <v>2026</v>
       </c>
       <c r="C218" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D218" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E218" s="1" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="F218" s="1" t="s">
         <v>361</v>
@@ -8500,7 +8539,7 @@
     </row>
     <row r="219" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A219" s="1" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B219" s="1">
         <v>2026</v>
@@ -8512,27 +8551,24 @@
         <v>265</v>
       </c>
       <c r="E219" s="1" t="s">
-        <v>372</v>
+        <v>231</v>
       </c>
       <c r="F219" s="1" t="s">
-        <v>262</v>
+        <v>361</v>
       </c>
       <c r="G219" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H219" s="1" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="I219" s="1">
-        <v>3</v>
-      </c>
-      <c r="J219" s="1">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="220" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A220" s="1" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B220" s="1">
         <v>2026</v>
@@ -8544,7 +8580,7 @@
         <v>265</v>
       </c>
       <c r="E220" s="1" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="F220" s="1" t="s">
         <v>361</v>
@@ -8556,7 +8592,7 @@
         <v>238</v>
       </c>
       <c r="I220" s="1">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="J220" s="1">
         <v>0</v>
@@ -8564,7 +8600,7 @@
     </row>
     <row r="221" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A221" s="1" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="B221" s="1">
         <v>2026</v>
@@ -8576,7 +8612,7 @@
         <v>265</v>
       </c>
       <c r="E221" s="1" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="F221" s="1" t="s">
         <v>361</v>
@@ -8588,7 +8624,7 @@
         <v>238</v>
       </c>
       <c r="I221" s="1">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="J221" s="1">
         <v>0</v>
@@ -8596,7 +8632,7 @@
     </row>
     <row r="222" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A222" s="1" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B222" s="1">
         <v>2026</v>
@@ -8608,19 +8644,19 @@
         <v>265</v>
       </c>
       <c r="E222" s="1" t="s">
-        <v>224</v>
+        <v>385</v>
       </c>
       <c r="F222" s="1" t="s">
-        <v>361</v>
+        <v>262</v>
       </c>
       <c r="G222" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H222" s="1" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="I222" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J222" s="1">
         <v>0</v>
@@ -8628,7 +8664,7 @@
     </row>
     <row r="223" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A223" s="1" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B223" s="1">
         <v>2026</v>
@@ -8640,7 +8676,7 @@
         <v>265</v>
       </c>
       <c r="E223" s="1" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="F223" s="1" t="s">
         <v>361</v>
@@ -8660,7 +8696,7 @@
     </row>
     <row r="224" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A224" s="1" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B224" s="1">
         <v>2026</v>
@@ -8672,19 +8708,19 @@
         <v>265</v>
       </c>
       <c r="E224" s="1" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="F224" s="1" t="s">
-        <v>262</v>
+        <v>361</v>
       </c>
       <c r="G224" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H224" s="1" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="I224" s="1">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="J224" s="1">
         <v>0</v>
@@ -8692,7 +8728,7 @@
     </row>
     <row r="225" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A225" s="1" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B225" s="1">
         <v>2026</v>
@@ -8704,19 +8740,19 @@
         <v>265</v>
       </c>
       <c r="E225" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F225" s="1" t="s">
-        <v>262</v>
+        <v>361</v>
       </c>
       <c r="G225" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H225" s="1" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="I225" s="1">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="J225" s="1">
         <v>0</v>
@@ -8724,28 +8760,28 @@
     </row>
     <row r="226" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A226" s="1" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B226" s="1">
         <v>2026</v>
       </c>
       <c r="C226" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D226" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E226" s="1" t="s">
-        <v>372</v>
+        <v>234</v>
       </c>
       <c r="F226" s="1" t="s">
-        <v>262</v>
+        <v>361</v>
       </c>
       <c r="G226" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H226" s="1" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="I226" s="1">
         <v>3</v>
@@ -8756,31 +8792,31 @@
     </row>
     <row r="227" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A227" s="1" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="B227" s="1">
         <v>2026</v>
       </c>
       <c r="C227" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D227" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E227" s="1" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="F227" s="1" t="s">
-        <v>361</v>
+        <v>262</v>
       </c>
       <c r="G227" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H227" s="1" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="I227" s="1">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="J227" s="1">
         <v>0</v>
@@ -8788,31 +8824,31 @@
     </row>
     <row r="228" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A228" s="1" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B228" s="1">
         <v>2026</v>
       </c>
       <c r="C228" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D228" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E228" s="1" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F228" s="1" t="s">
-        <v>361</v>
+        <v>262</v>
       </c>
       <c r="G228" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H228" s="1" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="I228" s="1">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="J228" s="1">
         <v>0</v>
@@ -8820,7 +8856,7 @@
     </row>
     <row r="229" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A229" s="1" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B229" s="1">
         <v>2026</v>
@@ -8832,7 +8868,7 @@
         <v>265</v>
       </c>
       <c r="E229" s="1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F229" s="1" t="s">
         <v>361</v>
@@ -8844,7 +8880,7 @@
         <v>238</v>
       </c>
       <c r="I229" s="1">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J229" s="1">
         <v>0</v>
@@ -8852,19 +8888,19 @@
     </row>
     <row r="230" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A230" s="1" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B230" s="1">
         <v>2026</v>
       </c>
       <c r="C230" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D230" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E230" s="1" t="s">
-        <v>224</v>
+        <v>385</v>
       </c>
       <c r="F230" s="1" t="s">
         <v>262</v>
@@ -8873,10 +8909,10 @@
         <v>368</v>
       </c>
       <c r="H230" s="1" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="I230" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J230" s="1">
         <v>0</v>
@@ -8884,7 +8920,7 @@
     </row>
     <row r="231" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A231" s="1" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B231" s="1">
         <v>2026</v>
@@ -8896,7 +8932,7 @@
         <v>265</v>
       </c>
       <c r="E231" s="1" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="F231" s="1" t="s">
         <v>361</v>
@@ -8908,7 +8944,7 @@
         <v>238</v>
       </c>
       <c r="I231" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J231" s="1">
         <v>0</v>
@@ -8916,7 +8952,7 @@
     </row>
     <row r="232" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A232" s="1" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B232" s="1">
         <v>2026</v>
@@ -8928,7 +8964,7 @@
         <v>265</v>
       </c>
       <c r="E232" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="F232" s="1" t="s">
         <v>361</v>
@@ -8940,7 +8976,7 @@
         <v>238</v>
       </c>
       <c r="I232" s="1">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J232" s="1">
         <v>0</v>
@@ -8948,7 +8984,7 @@
     </row>
     <row r="233" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A233" s="1" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="B233" s="1">
         <v>2026</v>
@@ -8960,7 +8996,7 @@
         <v>265</v>
       </c>
       <c r="E233" s="1" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="F233" s="1" t="s">
         <v>361</v>
@@ -8972,7 +9008,7 @@
         <v>238</v>
       </c>
       <c r="I233" s="1">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J233" s="1">
         <v>0</v>
@@ -8980,19 +9016,19 @@
     </row>
     <row r="234" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A234" s="1" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="B234" s="1">
         <v>2026</v>
       </c>
       <c r="C234" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D234" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E234" s="1" t="s">
-        <v>372</v>
+        <v>224</v>
       </c>
       <c r="F234" s="1" t="s">
         <v>262</v>
@@ -9001,10 +9037,10 @@
         <v>368</v>
       </c>
       <c r="H234" s="1" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="I234" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J234" s="1">
         <v>0</v>
@@ -9012,19 +9048,19 @@
     </row>
     <row r="235" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A235" s="1" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="B235" s="1">
         <v>2026</v>
       </c>
       <c r="C235" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D235" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E235" s="1" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="F235" s="1" t="s">
         <v>361</v>
@@ -9036,7 +9072,7 @@
         <v>238</v>
       </c>
       <c r="I235" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J235" s="1">
         <v>0</v>
@@ -9044,19 +9080,19 @@
     </row>
     <row r="236" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A236" s="1" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B236" s="1">
         <v>2026</v>
       </c>
       <c r="C236" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D236" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E236" s="1" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="F236" s="1" t="s">
         <v>361</v>
@@ -9068,7 +9104,7 @@
         <v>238</v>
       </c>
       <c r="I236" s="1">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J236" s="1">
         <v>0</v>
@@ -9076,19 +9112,19 @@
     </row>
     <row r="237" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A237" s="1" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B237" s="1">
         <v>2026</v>
       </c>
       <c r="C237" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D237" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E237" s="1" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="F237" s="1" t="s">
         <v>361</v>
@@ -9100,7 +9136,7 @@
         <v>238</v>
       </c>
       <c r="I237" s="1">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J237" s="1">
         <v>0</v>
@@ -9108,19 +9144,19 @@
     </row>
     <row r="238" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A238" s="1" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="B238" s="1">
         <v>2026</v>
       </c>
       <c r="C238" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D238" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E238" s="1" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="F238" s="1" t="s">
         <v>361</v>
@@ -9132,7 +9168,7 @@
         <v>238</v>
       </c>
       <c r="I238" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J238" s="1">
         <v>0</v>
@@ -9140,7 +9176,7 @@
     </row>
     <row r="239" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A239" s="1" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="B239" s="1">
         <v>2026</v>
@@ -9152,19 +9188,19 @@
         <v>265</v>
       </c>
       <c r="E239" s="1" t="s">
-        <v>234</v>
+        <v>385</v>
       </c>
       <c r="F239" s="1" t="s">
-        <v>361</v>
+        <v>262</v>
       </c>
       <c r="G239" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H239" s="1" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="I239" s="1">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J239" s="1">
         <v>0</v>
@@ -9172,31 +9208,31 @@
     </row>
     <row r="240" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A240" s="1" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B240" s="1">
         <v>2026</v>
       </c>
       <c r="C240" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D240" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E240" s="1" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="F240" s="1" t="s">
-        <v>262</v>
+        <v>361</v>
       </c>
       <c r="G240" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H240" s="1" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="I240" s="1">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="J240" s="1">
         <v>0</v>
@@ -9204,31 +9240,31 @@
     </row>
     <row r="241" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A241" s="1" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="B241" s="1">
         <v>2026</v>
       </c>
       <c r="C241" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D241" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E241" s="1" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="F241" s="1" t="s">
-        <v>262</v>
+        <v>361</v>
       </c>
       <c r="G241" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H241" s="1" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="I241" s="1">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="J241" s="1">
         <v>0</v>
@@ -9236,31 +9272,31 @@
     </row>
     <row r="242" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A242" s="1" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B242" s="1">
         <v>2026</v>
       </c>
       <c r="C242" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D242" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E242" s="1" t="s">
-        <v>372</v>
+        <v>232</v>
       </c>
       <c r="F242" s="1" t="s">
-        <v>262</v>
+        <v>361</v>
       </c>
       <c r="G242" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H242" s="1" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="I242" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J242" s="1">
         <v>0</v>
@@ -9268,19 +9304,19 @@
     </row>
     <row r="243" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A243" s="1" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="B243" s="1">
         <v>2026</v>
       </c>
       <c r="C243" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D243" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E243" s="1" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="F243" s="1" t="s">
         <v>361</v>
@@ -9292,7 +9328,7 @@
         <v>238</v>
       </c>
       <c r="I243" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J243" s="1">
         <v>0</v>
@@ -9300,19 +9336,19 @@
     </row>
     <row r="244" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A244" s="1" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B244" s="1">
         <v>2026</v>
       </c>
       <c r="C244" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D244" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E244" s="1" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="F244" s="1" t="s">
         <v>361</v>
@@ -9332,7 +9368,7 @@
     </row>
     <row r="245" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A245" s="1" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="B245" s="1">
         <v>2026</v>
@@ -9344,7 +9380,7 @@
         <v>265</v>
       </c>
       <c r="E245" s="1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F245" s="1" t="s">
         <v>361</v>
@@ -9356,7 +9392,7 @@
         <v>238</v>
       </c>
       <c r="I245" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J245" s="1">
         <v>0</v>
@@ -9364,7 +9400,7 @@
     </row>
     <row r="246" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A246" s="1" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B246" s="1">
         <v>2026</v>
@@ -9376,7 +9412,7 @@
         <v>265</v>
       </c>
       <c r="E246" s="1" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="F246" s="1" t="s">
         <v>262</v>
@@ -9385,10 +9421,10 @@
         <v>368</v>
       </c>
       <c r="H246" s="1" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="I246" s="1">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="J246" s="1">
         <v>0</v>
@@ -9396,31 +9432,31 @@
     </row>
     <row r="247" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A247" s="1" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B247" s="1">
         <v>2026</v>
       </c>
       <c r="C247" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D247" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E247" s="1" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="F247" s="1" t="s">
-        <v>361</v>
+        <v>262</v>
       </c>
       <c r="G247" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H247" s="1" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="I247" s="1">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="J247" s="1">
         <v>0</v>
@@ -9428,31 +9464,31 @@
     </row>
     <row r="248" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A248" s="1" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="B248" s="1">
         <v>2026</v>
       </c>
       <c r="C248" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D248" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E248" s="1" t="s">
-        <v>223</v>
+        <v>385</v>
       </c>
       <c r="F248" s="1" t="s">
-        <v>361</v>
+        <v>262</v>
       </c>
       <c r="G248" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H248" s="1" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="I248" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J248" s="1">
         <v>0</v>
@@ -9460,28 +9496,28 @@
     </row>
     <row r="249" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A249" s="1" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="B249" s="1">
         <v>2026</v>
       </c>
       <c r="C249" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D249" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E249" s="1" t="s">
-        <v>372</v>
+        <v>236</v>
       </c>
       <c r="F249" s="1" t="s">
-        <v>262</v>
+        <v>361</v>
       </c>
       <c r="G249" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H249" s="1" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="I249" s="1">
         <v>4</v>
@@ -9492,19 +9528,19 @@
     </row>
     <row r="250" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A250" s="1" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B250" s="1">
         <v>2026</v>
       </c>
       <c r="C250" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D250" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E250" s="1" t="s">
-        <v>236</v>
+        <v>226</v>
       </c>
       <c r="F250" s="1" t="s">
         <v>361</v>
@@ -9516,7 +9552,7 @@
         <v>238</v>
       </c>
       <c r="I250" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J250" s="1">
         <v>0</v>
@@ -9524,19 +9560,19 @@
     </row>
     <row r="251" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A251" s="1" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B251" s="1">
         <v>2026</v>
       </c>
       <c r="C251" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D251" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E251" s="1" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="F251" s="1" t="s">
         <v>361</v>
@@ -9556,28 +9592,28 @@
     </row>
     <row r="252" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A252" s="1" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="B252" s="1">
         <v>2026</v>
       </c>
       <c r="C252" s="1">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D252" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E252" s="1" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="F252" s="1" t="s">
-        <v>361</v>
+        <v>262</v>
       </c>
       <c r="G252" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H252" s="1" t="s">
-        <v>238</v>
+        <v>248</v>
       </c>
       <c r="I252" s="1">
         <v>3</v>
@@ -9588,7 +9624,7 @@
     </row>
     <row r="253" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A253" s="1" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="B253" s="1">
         <v>2026</v>
@@ -9600,7 +9636,7 @@
         <v>265</v>
       </c>
       <c r="E253" s="1" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="F253" s="1" t="s">
         <v>361</v>
@@ -9612,7 +9648,7 @@
         <v>238</v>
       </c>
       <c r="I253" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J253" s="1">
         <v>0</v>
@@ -9620,7 +9656,7 @@
     </row>
     <row r="254" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A254" s="1" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B254" s="1">
         <v>2026</v>
@@ -9632,19 +9668,19 @@
         <v>265</v>
       </c>
       <c r="E254" s="1" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="F254" s="1" t="s">
-        <v>262</v>
+        <v>361</v>
       </c>
       <c r="G254" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H254" s="1" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="I254" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="J254" s="1">
         <v>0</v>
@@ -9652,31 +9688,31 @@
     </row>
     <row r="255" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A255" s="1" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="B255" s="1">
         <v>2026</v>
       </c>
       <c r="C255" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D255" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E255" s="1" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="F255" s="1" t="s">
-        <v>262</v>
+        <v>361</v>
       </c>
       <c r="G255" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H255" s="1" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="I255" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="J255" s="1">
         <v>0</v>
@@ -9684,7 +9720,7 @@
     </row>
     <row r="256" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A256" s="1" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B256" s="1">
         <v>2026</v>
@@ -9696,19 +9732,19 @@
         <v>265</v>
       </c>
       <c r="E256" s="1" t="s">
-        <v>372</v>
+        <v>231</v>
       </c>
       <c r="F256" s="1" t="s">
-        <v>262</v>
+        <v>361</v>
       </c>
       <c r="G256" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H256" s="1" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="I256" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J256" s="1">
         <v>0</v>
@@ -9716,19 +9752,19 @@
     </row>
     <row r="257" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A257" s="1" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="B257" s="1">
         <v>2026</v>
       </c>
       <c r="C257" s="1">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D257" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E257" s="1" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="F257" s="1" t="s">
         <v>361</v>
@@ -9740,7 +9776,7 @@
         <v>238</v>
       </c>
       <c r="I257" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J257" s="1">
         <v>0</v>
@@ -9748,19 +9784,19 @@
     </row>
     <row r="258" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A258" s="1" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="B258" s="1">
         <v>2026</v>
       </c>
       <c r="C258" s="1">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D258" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E258" s="1" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="F258" s="1" t="s">
         <v>361</v>
@@ -9772,7 +9808,7 @@
         <v>238</v>
       </c>
       <c r="I258" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J258" s="1">
         <v>0</v>
@@ -9780,31 +9816,31 @@
     </row>
     <row r="259" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A259" s="1" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="B259" s="1">
         <v>2026</v>
       </c>
       <c r="C259" s="1">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D259" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E259" s="1" t="s">
-        <v>232</v>
+        <v>385</v>
       </c>
       <c r="F259" s="1" t="s">
-        <v>361</v>
+        <v>262</v>
       </c>
       <c r="G259" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H259" s="1" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="I259" s="1">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J259" s="1">
         <v>0</v>
@@ -9812,31 +9848,31 @@
     </row>
     <row r="260" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A260" s="1" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B260" s="1">
         <v>2026</v>
       </c>
       <c r="C260" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D260" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E260" s="1" t="s">
-        <v>224</v>
+        <v>236</v>
       </c>
       <c r="F260" s="1" t="s">
-        <v>262</v>
+        <v>361</v>
       </c>
       <c r="G260" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H260" s="1" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="I260" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J260" s="1">
         <v>0</v>
@@ -9844,19 +9880,19 @@
     </row>
     <row r="261" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A261" s="1" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="B261" s="1">
         <v>2026</v>
       </c>
       <c r="C261" s="1">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D261" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E261" s="1" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="F261" s="1" t="s">
         <v>361</v>
@@ -9876,19 +9912,19 @@
     </row>
     <row r="262" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A262" s="1" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="B262" s="1">
         <v>2026</v>
       </c>
       <c r="C262" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D262" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E262" s="1" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="F262" s="1" t="s">
         <v>361</v>
@@ -9900,7 +9936,7 @@
         <v>238</v>
       </c>
       <c r="I262" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J262" s="1">
         <v>0</v>
@@ -9908,19 +9944,19 @@
     </row>
     <row r="263" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A263" s="1" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="B263" s="1">
         <v>2026</v>
       </c>
       <c r="C263" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D263" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E263" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F263" s="1" t="s">
         <v>361</v>
@@ -9932,7 +9968,7 @@
         <v>238</v>
       </c>
       <c r="I263" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J263" s="1">
         <v>0</v>
@@ -9940,19 +9976,19 @@
     </row>
     <row r="264" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A264" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="B264" s="1">
         <v>2026</v>
       </c>
       <c r="C264" s="1">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D264" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E264" s="1" t="s">
-        <v>372</v>
+        <v>228</v>
       </c>
       <c r="F264" s="1" t="s">
         <v>262</v>
@@ -9961,10 +9997,10 @@
         <v>368</v>
       </c>
       <c r="H264" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="I264" s="1">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="J264" s="1">
         <v>0</v>
@@ -9972,31 +10008,31 @@
     </row>
     <row r="265" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A265" s="1" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="B265" s="1">
         <v>2026</v>
       </c>
       <c r="C265" s="1">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D265" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E265" s="1" t="s">
-        <v>236</v>
+        <v>223</v>
       </c>
       <c r="F265" s="1" t="s">
-        <v>361</v>
+        <v>262</v>
       </c>
       <c r="G265" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H265" s="1" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="I265" s="1">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="J265" s="1">
         <v>0</v>
@@ -10004,31 +10040,31 @@
     </row>
     <row r="266" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A266" s="1" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="B266" s="1">
         <v>2026</v>
       </c>
       <c r="C266" s="1">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D266" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E266" s="1" t="s">
-        <v>226</v>
+        <v>385</v>
       </c>
       <c r="F266" s="1" t="s">
-        <v>361</v>
+        <v>262</v>
       </c>
       <c r="G266" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H266" s="1" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="I266" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J266" s="1">
         <v>0</v>
@@ -10036,19 +10072,19 @@
     </row>
     <row r="267" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A267" s="1" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B267" s="1">
         <v>2026</v>
       </c>
       <c r="C267" s="1">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D267" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E267" s="1" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="F267" s="1" t="s">
         <v>361</v>
@@ -10060,7 +10096,7 @@
         <v>238</v>
       </c>
       <c r="I267" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J267" s="1">
         <v>0</v>
@@ -10068,19 +10104,19 @@
     </row>
     <row r="268" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A268" s="1" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="B268" s="1">
         <v>2026</v>
       </c>
       <c r="C268" s="1">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D268" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E268" s="1" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F268" s="1" t="s">
         <v>361</v>
@@ -10092,7 +10128,7 @@
         <v>238</v>
       </c>
       <c r="I268" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J268" s="1">
         <v>0</v>
@@ -10100,19 +10136,19 @@
     </row>
     <row r="269" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A269" s="1" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B269" s="1">
         <v>2026</v>
       </c>
       <c r="C269" s="1">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D269" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E269" s="1" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="F269" s="1" t="s">
         <v>361</v>
@@ -10124,7 +10160,7 @@
         <v>238</v>
       </c>
       <c r="I269" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J269" s="1">
         <v>0</v>
@@ -10132,19 +10168,19 @@
     </row>
     <row r="270" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A270" s="1" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B270" s="1">
         <v>2026</v>
       </c>
       <c r="C270" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D270" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E270" s="1" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="F270" s="1" t="s">
         <v>262</v>
@@ -10153,10 +10189,10 @@
         <v>368</v>
       </c>
       <c r="H270" s="1" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="I270" s="1">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="J270" s="1">
         <v>0</v>
@@ -10164,31 +10200,31 @@
     </row>
     <row r="271" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A271" s="1" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="B271" s="1">
         <v>2026</v>
       </c>
       <c r="C271" s="1">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D271" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E271" s="1" t="s">
-        <v>223</v>
+        <v>234</v>
       </c>
       <c r="F271" s="1" t="s">
-        <v>262</v>
+        <v>361</v>
       </c>
       <c r="G271" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H271" s="1" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="I271" s="1">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="J271" s="1">
         <v>0</v>
@@ -10196,31 +10232,31 @@
     </row>
     <row r="272" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A272" s="1" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B272" s="1">
         <v>2026</v>
       </c>
       <c r="C272" s="1">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D272" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E272" s="1" t="s">
-        <v>372</v>
+        <v>228</v>
       </c>
       <c r="F272" s="1" t="s">
-        <v>262</v>
+        <v>361</v>
       </c>
       <c r="G272" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H272" s="1" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="I272" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J272" s="1">
         <v>0</v>
@@ -10228,19 +10264,19 @@
     </row>
     <row r="273" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A273" s="1" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="B273" s="1">
         <v>2026</v>
       </c>
       <c r="C273" s="1">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D273" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E273" s="1" t="s">
-        <v>236</v>
+        <v>223</v>
       </c>
       <c r="F273" s="1" t="s">
         <v>361</v>
@@ -10252,7 +10288,7 @@
         <v>238</v>
       </c>
       <c r="I273" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J273" s="1">
         <v>0</v>
@@ -10260,31 +10296,31 @@
     </row>
     <row r="274" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A274" s="1" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="B274" s="1">
         <v>2026</v>
       </c>
       <c r="C274" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D274" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E274" s="1" t="s">
-        <v>226</v>
+        <v>385</v>
       </c>
       <c r="F274" s="1" t="s">
-        <v>361</v>
+        <v>262</v>
       </c>
       <c r="G274" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H274" s="1" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="I274" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J274" s="1">
         <v>0</v>
@@ -10292,19 +10328,19 @@
     </row>
     <row r="275" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A275" s="1" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="B275" s="1">
         <v>2026</v>
       </c>
       <c r="C275" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D275" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E275" s="1" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="F275" s="1" t="s">
         <v>361</v>
@@ -10316,7 +10352,7 @@
         <v>238</v>
       </c>
       <c r="I275" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J275" s="1">
         <v>0</v>
@@ -10324,31 +10360,31 @@
     </row>
     <row r="276" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A276" s="1" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B276" s="1">
         <v>2026</v>
       </c>
       <c r="C276" s="1">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D276" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E276" s="1" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F276" s="1" t="s">
-        <v>262</v>
+        <v>361</v>
       </c>
       <c r="G276" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H276" s="1" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="I276" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J276" s="1">
         <v>0</v>
@@ -10356,19 +10392,19 @@
     </row>
     <row r="277" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A277" s="1" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="B277" s="1">
         <v>2026</v>
       </c>
       <c r="C277" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D277" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E277" s="1" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="F277" s="1" t="s">
         <v>361</v>
@@ -10380,7 +10416,7 @@
         <v>238</v>
       </c>
       <c r="I277" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J277" s="1">
         <v>0</v>
@@ -10388,19 +10424,19 @@
     </row>
     <row r="278" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A278" s="1" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="B278" s="1">
         <v>2026</v>
       </c>
       <c r="C278" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D278" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E278" s="1" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="F278" s="1" t="s">
         <v>361</v>
@@ -10412,7 +10448,7 @@
         <v>238</v>
       </c>
       <c r="I278" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J278" s="1">
         <v>0</v>
@@ -10420,19 +10456,19 @@
     </row>
     <row r="279" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A279" s="1" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="B279" s="1">
         <v>2026</v>
       </c>
       <c r="C279" s="1">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D279" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E279" s="1" t="s">
-        <v>223</v>
+        <v>234</v>
       </c>
       <c r="F279" s="1" t="s">
         <v>361</v>
@@ -10444,7 +10480,7 @@
         <v>238</v>
       </c>
       <c r="I279" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J279" s="1">
         <v>0</v>
@@ -10452,31 +10488,31 @@
     </row>
     <row r="280" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A280" s="1" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B280" s="1">
         <v>2026</v>
       </c>
       <c r="C280" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D280" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E280" s="1" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="F280" s="1" t="s">
-        <v>361</v>
+        <v>262</v>
       </c>
       <c r="G280" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H280" s="1" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="I280" s="1">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="J280" s="1">
         <v>0</v>
@@ -10484,31 +10520,31 @@
     </row>
     <row r="281" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A281" s="1" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="B281" s="1">
         <v>2026</v>
       </c>
       <c r="C281" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D281" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E281" s="1" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="F281" s="1" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="G281" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H281" s="1" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I281" s="1">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="J281" s="1">
         <v>0</v>
@@ -10516,19 +10552,19 @@
     </row>
     <row r="282" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A282" s="1" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B282" s="1">
         <v>2026</v>
       </c>
       <c r="C282" s="1">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D282" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E282" s="1" t="s">
-        <v>228</v>
+        <v>385</v>
       </c>
       <c r="F282" s="1" t="s">
         <v>262</v>
@@ -10537,10 +10573,10 @@
         <v>368</v>
       </c>
       <c r="H282" s="1" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="I282" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="J282" s="1">
         <v>0</v>
@@ -10548,31 +10584,31 @@
     </row>
     <row r="283" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A283" s="1" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B283" s="1">
         <v>2026</v>
       </c>
       <c r="C283" s="1">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D283" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E283" s="1" t="s">
-        <v>223</v>
+        <v>236</v>
       </c>
       <c r="F283" s="1" t="s">
-        <v>262</v>
+        <v>361</v>
       </c>
       <c r="G283" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H283" s="1" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="I283" s="1">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="J283" s="1">
         <v>0</v>
@@ -10580,31 +10616,31 @@
     </row>
     <row r="284" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A284" s="1" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="B284" s="1">
         <v>2026</v>
       </c>
       <c r="C284" s="1">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D284" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E284" s="1" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F284" s="1" t="s">
-        <v>262</v>
+        <v>361</v>
       </c>
       <c r="G284" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H284" s="1" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="I284" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J284" s="1">
         <v>0</v>
@@ -10612,19 +10648,19 @@
     </row>
     <row r="285" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A285" s="1" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="B285" s="1">
         <v>2026</v>
       </c>
       <c r="C285" s="1">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D285" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E285" s="1" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="F285" s="1" t="s">
         <v>361</v>
@@ -10636,7 +10672,7 @@
         <v>238</v>
       </c>
       <c r="I285" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J285" s="1">
         <v>0</v>
@@ -10644,31 +10680,31 @@
     </row>
     <row r="286" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A286" s="1" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="B286" s="1">
         <v>2026</v>
       </c>
       <c r="C286" s="1">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D286" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E286" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F286" s="1" t="s">
-        <v>361</v>
+        <v>262</v>
       </c>
       <c r="G286" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H286" s="1" t="s">
-        <v>238</v>
+        <v>248</v>
       </c>
       <c r="I286" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J286" s="1">
         <v>0</v>
@@ -10676,19 +10712,19 @@
     </row>
     <row r="287" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A287" s="1" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B287" s="1">
         <v>2026</v>
       </c>
       <c r="C287" s="1">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D287" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E287" s="1" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="F287" s="1" t="s">
         <v>361</v>
@@ -10700,7 +10736,7 @@
         <v>238</v>
       </c>
       <c r="I287" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J287" s="1">
         <v>0</v>
@@ -10708,13 +10744,13 @@
     </row>
     <row r="288" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A288" s="1" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="B288" s="1">
         <v>2026</v>
       </c>
       <c r="C288" s="1">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D288" s="1" t="s">
         <v>265</v>
@@ -10723,16 +10759,16 @@
         <v>228</v>
       </c>
       <c r="F288" s="1" t="s">
-        <v>262</v>
+        <v>361</v>
       </c>
       <c r="G288" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H288" s="1" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="I288" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="J288" s="1">
         <v>0</v>
@@ -10740,13 +10776,13 @@
     </row>
     <row r="289" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A289" s="1" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="B289" s="1">
         <v>2026</v>
       </c>
       <c r="C289" s="1">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D289" s="1" t="s">
         <v>265</v>
@@ -10755,16 +10791,16 @@
         <v>223</v>
       </c>
       <c r="F289" s="1" t="s">
-        <v>262</v>
+        <v>361</v>
       </c>
       <c r="G289" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H289" s="1" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="I289" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="J289" s="1">
         <v>0</v>
@@ -10772,13 +10808,13 @@
     </row>
     <row r="290" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A290" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="B290" s="1">
         <v>2026</v>
       </c>
       <c r="C290" s="1">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D290" s="1" t="s">
         <v>265</v>
@@ -10787,16 +10823,16 @@
         <v>224</v>
       </c>
       <c r="F290" s="1" t="s">
-        <v>262</v>
+        <v>361</v>
       </c>
       <c r="G290" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H290" s="1" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="I290" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J290" s="1">
         <v>0</v>
@@ -10804,13 +10840,13 @@
     </row>
     <row r="291" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A291" s="1" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="B291" s="1">
         <v>2026</v>
       </c>
       <c r="C291" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D291" s="1" t="s">
         <v>265</v>
@@ -10828,7 +10864,7 @@
         <v>242</v>
       </c>
       <c r="I291" s="1">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="J291" s="1">
         <v>0</v>
@@ -10836,13 +10872,13 @@
     </row>
     <row r="292" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A292" s="1" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B292" s="1">
         <v>2026</v>
       </c>
       <c r="C292" s="1">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D292" s="1" t="s">
         <v>265</v>
@@ -10851,16 +10887,16 @@
         <v>228</v>
       </c>
       <c r="F292" s="1" t="s">
-        <v>361</v>
+        <v>262</v>
       </c>
       <c r="G292" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H292" s="1" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="I292" s="1">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="J292" s="1">
         <v>0</v>
@@ -10868,13 +10904,13 @@
     </row>
     <row r="293" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A293" s="1" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="B293" s="1">
         <v>2026</v>
       </c>
       <c r="C293" s="1">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D293" s="1" t="s">
         <v>265</v>
@@ -10883,16 +10919,16 @@
         <v>223</v>
       </c>
       <c r="F293" s="1" t="s">
-        <v>361</v>
+        <v>262</v>
       </c>
       <c r="G293" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H293" s="1" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="I293" s="1">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="J293" s="1">
         <v>0</v>
@@ -10900,13 +10936,13 @@
     </row>
     <row r="294" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A294" s="1" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B294" s="1">
         <v>2026</v>
       </c>
       <c r="C294" s="1">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D294" s="1" t="s">
         <v>265</v>
@@ -10915,16 +10951,16 @@
         <v>224</v>
       </c>
       <c r="F294" s="1" t="s">
-        <v>361</v>
+        <v>262</v>
       </c>
       <c r="G294" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H294" s="1" t="s">
-        <v>238</v>
+        <v>248</v>
       </c>
       <c r="I294" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J294" s="1">
         <v>0</v>
@@ -10932,7 +10968,7 @@
     </row>
     <row r="295" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A295" s="1" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B295" s="1">
         <v>2026</v>
@@ -10944,7 +10980,7 @@
         <v>265</v>
       </c>
       <c r="E295" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="F295" s="1" t="s">
         <v>361</v>
@@ -10956,7 +10992,7 @@
         <v>238</v>
       </c>
       <c r="I295" s="1">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="J295" s="1">
         <v>0</v>
@@ -10964,31 +11000,31 @@
     </row>
     <row r="296" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A296" s="1" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B296" s="1">
         <v>2026</v>
       </c>
       <c r="C296" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D296" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E296" s="1" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="F296" s="1" t="s">
-        <v>263</v>
+        <v>361</v>
       </c>
       <c r="G296" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H296" s="1" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="I296" s="1">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J296" s="1">
         <v>0</v>
@@ -10996,31 +11032,31 @@
     </row>
     <row r="297" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A297" s="1" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="B297" s="1">
         <v>2026</v>
       </c>
       <c r="C297" s="1">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D297" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E297" s="1" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="F297" s="1" t="s">
-        <v>262</v>
+        <v>361</v>
       </c>
       <c r="G297" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H297" s="1" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="I297" s="1">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="J297" s="1">
         <v>0</v>
@@ -11028,19 +11064,19 @@
     </row>
     <row r="298" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A298" s="1" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B298" s="1">
         <v>2026</v>
       </c>
       <c r="C298" s="1">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D298" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E298" s="1" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="F298" s="1" t="s">
         <v>262</v>
@@ -11049,7 +11085,7 @@
         <v>368</v>
       </c>
       <c r="H298" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="I298" s="1">
         <v>12</v>
@@ -11060,19 +11096,19 @@
     </row>
     <row r="299" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A299" s="1" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="B299" s="1">
         <v>2026</v>
       </c>
       <c r="C299" s="1">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D299" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E299" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F299" s="1" t="s">
         <v>262</v>
@@ -11081,10 +11117,10 @@
         <v>368</v>
       </c>
       <c r="H299" s="1" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="I299" s="1">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="J299" s="1">
         <v>0</v>
@@ -11092,7 +11128,7 @@
     </row>
     <row r="300" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A300" s="1" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="B300" s="1">
         <v>2026</v>
@@ -11104,19 +11140,19 @@
         <v>265</v>
       </c>
       <c r="E300" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="F300" s="1" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G300" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H300" s="1" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="I300" s="1">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="J300" s="1">
         <v>0</v>
@@ -11124,31 +11160,31 @@
     </row>
     <row r="301" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A301" s="1" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="B301" s="1">
         <v>2026</v>
       </c>
       <c r="C301" s="1">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D301" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E301" s="1" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F301" s="1" t="s">
-        <v>361</v>
+        <v>263</v>
       </c>
       <c r="G301" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H301" s="1" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I301" s="1">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J301" s="1">
         <v>0</v>
@@ -11156,19 +11192,19 @@
     </row>
     <row r="302" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A302" s="1" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B302" s="1">
         <v>2026</v>
       </c>
       <c r="C302" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D302" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E302" s="1" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="F302" s="1" t="s">
         <v>361</v>
@@ -11188,19 +11224,19 @@
     </row>
     <row r="303" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A303" s="1" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B303" s="1">
         <v>2026</v>
       </c>
       <c r="C303" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D303" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E303" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F303" s="1" t="s">
         <v>361</v>
@@ -11212,7 +11248,7 @@
         <v>238</v>
       </c>
       <c r="I303" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J303" s="1">
         <v>0</v>
@@ -11220,7 +11256,7 @@
     </row>
     <row r="304" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A304" s="1" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B304" s="1">
         <v>2026</v>
@@ -11232,19 +11268,19 @@
         <v>265</v>
       </c>
       <c r="E304" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="F304" s="1" t="s">
-        <v>264</v>
+        <v>361</v>
       </c>
       <c r="G304" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H304" s="1" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="I304" s="1">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="J304" s="1">
         <v>0</v>
@@ -11252,31 +11288,31 @@
     </row>
     <row r="305" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A305" s="1" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="B305" s="1">
         <v>2026</v>
       </c>
       <c r="C305" s="1">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D305" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E305" s="1" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="F305" s="1" t="s">
-        <v>263</v>
+        <v>361</v>
       </c>
       <c r="G305" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H305" s="1" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="I305" s="1">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="J305" s="1">
         <v>0</v>
@@ -11284,31 +11320,31 @@
     </row>
     <row r="306" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A306" s="1" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B306" s="1">
         <v>2026</v>
       </c>
       <c r="C306" s="1">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D306" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E306" s="1" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F306" s="1" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="G306" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H306" s="1" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="I306" s="1">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J306" s="1">
         <v>0</v>
@@ -11316,19 +11352,19 @@
     </row>
     <row r="307" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A307" s="1" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="B307" s="1">
         <v>2026</v>
       </c>
       <c r="C307" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D307" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E307" s="1" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="F307" s="1" t="s">
         <v>262</v>
@@ -11337,7 +11373,7 @@
         <v>368</v>
       </c>
       <c r="H307" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="I307" s="1">
         <v>12</v>
@@ -11348,19 +11384,19 @@
     </row>
     <row r="308" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A308" s="1" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B308" s="1">
         <v>2026</v>
       </c>
       <c r="C308" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D308" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E308" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F308" s="1" t="s">
         <v>262</v>
@@ -11369,10 +11405,10 @@
         <v>368</v>
       </c>
       <c r="H308" s="1" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="I308" s="1">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="J308" s="1">
         <v>0</v>
@@ -11380,31 +11416,31 @@
     </row>
     <row r="309" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A309" s="1" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B309" s="1">
         <v>2026</v>
       </c>
       <c r="C309" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D309" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E309" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="F309" s="1" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G309" s="1" t="s">
         <v>368</v>
       </c>
       <c r="H309" s="1" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="I309" s="1">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="J309" s="1">
         <v>0</v>
@@ -11412,38 +11448,454 @@
     </row>
     <row r="310" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A310" s="1" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="B310" s="1">
         <v>2026</v>
       </c>
       <c r="C310" s="1">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D310" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E310" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="F310" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="G310" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="H310" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="I310" s="1">
+        <v>6</v>
+      </c>
+      <c r="J310" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="311" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A311" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="B311" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C311" s="1">
+        <v>12</v>
+      </c>
+      <c r="D311" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="E311" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="F311" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="G311" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="H311" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="I311" s="1">
+        <v>6</v>
+      </c>
+      <c r="J311" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="312" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A312" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="B312" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C312" s="1">
+        <v>12</v>
+      </c>
+      <c r="D312" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="E312" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="F312" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="G312" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="H312" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="I312" s="1">
+        <v>6</v>
+      </c>
+      <c r="J312" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="313" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A313" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="B313" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C313" s="1">
+        <v>12</v>
+      </c>
+      <c r="D313" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="E313" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="F313" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="G313" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="H313" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="I313" s="1">
+        <v>4</v>
+      </c>
+      <c r="J313" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="314" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A314" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="B314" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C314" s="1">
+        <v>11</v>
+      </c>
+      <c r="D314" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="E314" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="F314" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="G314" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="H314" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="I314" s="1">
+        <v>6</v>
+      </c>
+      <c r="J314" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="315" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A315" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="B315" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C315" s="1">
+        <v>11</v>
+      </c>
+      <c r="D315" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="E315" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="F310" s="1" t="s">
+      <c r="F315" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="G310" s="1" t="s">
-        <v>368</v>
-      </c>
-      <c r="H310" s="1" t="s">
+      <c r="G315" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="H315" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="I310" s="1">
+      <c r="I315" s="1">
+        <v>10</v>
+      </c>
+      <c r="J315" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="316" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A316" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="B316" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C316" s="1">
+        <v>12</v>
+      </c>
+      <c r="D316" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="E316" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="F316" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="G316" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="H316" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="I316" s="1">
+        <v>12</v>
+      </c>
+      <c r="J316" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="317" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A317" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="B317" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C317" s="1">
+        <v>12</v>
+      </c>
+      <c r="D317" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="E317" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="F317" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="G317" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="H317" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="I317" s="1">
+        <v>12</v>
+      </c>
+      <c r="J317" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="318" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A318" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="B318" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C318" s="1">
+        <v>12</v>
+      </c>
+      <c r="D318" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="E318" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="F318" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="G318" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="H318" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="I318" s="1">
+        <v>4</v>
+      </c>
+      <c r="J318" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="319" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A319" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="B319" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C319" s="1">
+        <v>12</v>
+      </c>
+      <c r="D319" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="E319" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="F319" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="G319" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="H319" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="I319" s="1">
+        <v>6</v>
+      </c>
+      <c r="J319" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="320" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A320" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="B320" s="1">
+        <v>2027</v>
+      </c>
+      <c r="C320" s="1">
         <v>1</v>
       </c>
-      <c r="J310" s="1">
+      <c r="D320" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="E320" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="F320" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="G320" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="H320" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="I320" s="1">
+        <v>6</v>
+      </c>
+      <c r="J320" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="321" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A321" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="B321" s="1">
+        <v>2027</v>
+      </c>
+      <c r="C321" s="1">
+        <v>2</v>
+      </c>
+      <c r="D321" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="E321" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="F321" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="G321" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="H321" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="I321" s="1">
+        <v>6</v>
+      </c>
+      <c r="J321" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="322" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A322" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="B322" s="1">
+        <v>2027</v>
+      </c>
+      <c r="C322" s="1">
+        <v>3</v>
+      </c>
+      <c r="D322" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="E322" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="F322" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="G322" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="H322" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="I322" s="1">
+        <v>6</v>
+      </c>
+      <c r="J322" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="323" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A323" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="B323" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C323" s="1">
+        <v>12</v>
+      </c>
+      <c r="D323" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="E323" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="F323" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="G323" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="H323" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="I323" s="1">
+        <v>10</v>
+      </c>
+      <c r="J323" s="1">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J310" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:J323" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
update metas (new cas)
</commit_message>
<xml_diff>
--- a/data/metas.xlsx
+++ b/data/metas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROYECTOS - 2026 (DEV)\DEV - POI\Insights_POI\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BDCD5D2-A014-4A57-BA46-9AFEDA4751FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1962483B-9673-4C56-87BD-B5ACF3953DF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,6 +33,69 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={67BB8CD7-6C9F-486E-9D3E-D96EE5626E58}</author>
+    <author>tc={5C39EC35-44CB-4DBF-8FA1-F5DD38C0E19A}</author>
+    <author>tc={F21B41F8-36BB-4871-A2E3-DC15F64BF9DE}</author>
+    <author>tc={B7004EAA-2AD6-442B-AF75-E000AC90D04C}</author>
+    <author>tc={FD84FD04-E8AC-47F4-AECE-E00404C82C88}</author>
+    <author>tc={FD8921CA-58D6-4D39-9CBE-343EB1D00BAA}</author>
+  </authors>
+  <commentList>
+    <comment ref="I97" authorId="0" shapeId="0" xr:uid="{67BB8CD7-6C9F-486E-9D3E-D96EE5626E58}">
+      <text>
+        <t>[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    4 con erika</t>
+      </text>
+    </comment>
+    <comment ref="I102" authorId="1" shapeId="0" xr:uid="{5C39EC35-44CB-4DBF-8FA1-F5DD38C0E19A}">
+      <text>
+        <t>[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    3 con erika</t>
+      </text>
+    </comment>
+    <comment ref="I113" authorId="2" shapeId="0" xr:uid="{F21B41F8-36BB-4871-A2E3-DC15F64BF9DE}">
+      <text>
+        <t>[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    15 con erika</t>
+      </text>
+    </comment>
+    <comment ref="I167" authorId="3" shapeId="0" xr:uid="{B7004EAA-2AD6-442B-AF75-E000AC90D04C}">
+      <text>
+        <t>[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    5 con erika</t>
+      </text>
+    </comment>
+    <comment ref="I190" authorId="4" shapeId="0" xr:uid="{FD84FD04-E8AC-47F4-AECE-E00404C82C88}">
+      <text>
+        <t>[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    2 con erika</t>
+      </text>
+    </comment>
+    <comment ref="I206" authorId="5" shapeId="0" xr:uid="{FD8921CA-58D6-4D39-9CBE-343EB1D00BAA}">
+      <text>
+        <t>[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    3 con erika</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1972" uniqueCount="393">
   <si>
@@ -1219,7 +1282,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1249,6 +1312,12 @@
       <sz val="12"/>
       <color theme="9" tint="-0.249977111117893"/>
       <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -1292,6 +1361,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Instituto Tecnológico de la Producción" id="{D9166656-C808-4125-A906-92544B2BCC6F}" userId="e413a67a96bae1e1" providerId="Windows Live"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1579,8 +1654,32 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="I97" dT="2026-07-10T15:00:26.16" personId="{D9166656-C808-4125-A906-92544B2BCC6F}" id="{67BB8CD7-6C9F-486E-9D3E-D96EE5626E58}">
+    <text>4 con erika</text>
+  </threadedComment>
+  <threadedComment ref="I102" dT="2026-07-10T15:00:33.14" personId="{D9166656-C808-4125-A906-92544B2BCC6F}" id="{5C39EC35-44CB-4DBF-8FA1-F5DD38C0E19A}">
+    <text>3 con erika</text>
+  </threadedComment>
+  <threadedComment ref="I113" dT="2026-07-10T15:00:14.23" personId="{D9166656-C808-4125-A906-92544B2BCC6F}" id="{F21B41F8-36BB-4871-A2E3-DC15F64BF9DE}">
+    <text>15 con erika</text>
+  </threadedComment>
+  <threadedComment ref="I167" dT="2026-07-10T15:00:40.67" personId="{D9166656-C808-4125-A906-92544B2BCC6F}" id="{B7004EAA-2AD6-442B-AF75-E000AC90D04C}">
+    <text>5 con erika</text>
+  </threadedComment>
+  <threadedComment ref="I190" dT="2026-07-10T15:00:50.31" personId="{D9166656-C808-4125-A906-92544B2BCC6F}" id="{FD84FD04-E8AC-47F4-AECE-E00404C82C88}">
+    <text>2 con erika</text>
+  </threadedComment>
+  <threadedComment ref="I206" dT="2026-07-10T15:00:57.19" personId="{D9166656-C808-4125-A906-92544B2BCC6F}" id="{FD8921CA-58D6-4D39-9CBE-343EB1D00BAA}">
+    <text>3 con erika</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:J328"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1660,7 +1759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -1692,7 +1791,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -1724,7 +1823,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
@@ -1756,7 +1855,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -1788,7 +1887,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -1820,7 +1919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>15</v>
       </c>
@@ -1852,7 +1951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
@@ -1884,7 +1983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>17</v>
       </c>
@@ -1916,7 +2015,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>18</v>
       </c>
@@ -1948,7 +2047,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>19</v>
       </c>
@@ -1980,7 +2079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>20</v>
       </c>
@@ -2012,7 +2111,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>21</v>
       </c>
@@ -2044,7 +2143,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>22</v>
       </c>
@@ -2076,7 +2175,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>23</v>
       </c>
@@ -2108,7 +2207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>24</v>
       </c>
@@ -2140,7 +2239,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>25</v>
       </c>
@@ -2204,7 +2303,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>27</v>
       </c>
@@ -2236,7 +2335,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>28</v>
       </c>
@@ -2268,7 +2367,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>29</v>
       </c>
@@ -2300,7 +2399,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>30</v>
       </c>
@@ -2364,7 +2463,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>32</v>
       </c>
@@ -2396,7 +2495,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>33</v>
       </c>
@@ -2428,7 +2527,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>34</v>
       </c>
@@ -2460,7 +2559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>35</v>
       </c>
@@ -2492,7 +2591,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>36</v>
       </c>
@@ -2524,7 +2623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>37</v>
       </c>
@@ -2556,7 +2655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>38</v>
       </c>
@@ -2588,7 +2687,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>39</v>
       </c>
@@ -2620,7 +2719,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>40</v>
       </c>
@@ -2652,7 +2751,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>41</v>
       </c>
@@ -2684,7 +2783,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>42</v>
       </c>
@@ -2716,7 +2815,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>43</v>
       </c>
@@ -2748,7 +2847,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>44</v>
       </c>
@@ -2780,7 +2879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>45</v>
       </c>
@@ -2812,7 +2911,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>46</v>
       </c>
@@ -2876,7 +2975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>48</v>
       </c>
@@ -2908,7 +3007,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>49</v>
       </c>
@@ -2940,7 +3039,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>50</v>
       </c>
@@ -2972,7 +3071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>51</v>
       </c>
@@ -3004,7 +3103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>52</v>
       </c>
@@ -3036,7 +3135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>53</v>
       </c>
@@ -3068,7 +3167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>54</v>
       </c>
@@ -3100,7 +3199,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>55</v>
       </c>
@@ -3132,7 +3231,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>56</v>
       </c>
@@ -3164,7 +3263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>57</v>
       </c>
@@ -3196,7 +3295,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>58</v>
       </c>
@@ -3260,7 +3359,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>60</v>
       </c>
@@ -3292,7 +3391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>61</v>
       </c>
@@ -3324,7 +3423,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>62</v>
       </c>
@@ -3356,7 +3455,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>63</v>
       </c>
@@ -3388,7 +3487,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>64</v>
       </c>
@@ -3420,7 +3519,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>65</v>
       </c>
@@ -3452,7 +3551,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>66</v>
       </c>
@@ -3484,7 +3583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>67</v>
       </c>
@@ -3516,7 +3615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>68</v>
       </c>
@@ -3548,7 +3647,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>69</v>
       </c>
@@ -3580,7 +3679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>70</v>
       </c>
@@ -3612,7 +3711,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>71</v>
       </c>
@@ -3644,7 +3743,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>72</v>
       </c>
@@ -3676,7 +3775,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>73</v>
       </c>
@@ -3708,7 +3807,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>74</v>
       </c>
@@ -3740,7 +3839,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>75</v>
       </c>
@@ -3772,7 +3871,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>76</v>
       </c>
@@ -3804,7 +3903,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>77</v>
       </c>
@@ -3836,7 +3935,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>78</v>
       </c>
@@ -3868,7 +3967,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>79</v>
       </c>
@@ -3932,7 +4031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>81</v>
       </c>
@@ -3964,7 +4063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>82</v>
       </c>
@@ -3996,7 +4095,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>83</v>
       </c>
@@ -4028,7 +4127,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>84</v>
       </c>
@@ -4060,7 +4159,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>85</v>
       </c>
@@ -4092,7 +4191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>86</v>
       </c>
@@ -4124,7 +4223,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>87</v>
       </c>
@@ -4156,7 +4255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>88</v>
       </c>
@@ -4188,7 +4287,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>89</v>
       </c>
@@ -4220,7 +4319,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>90</v>
       </c>
@@ -4252,7 +4351,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>91</v>
       </c>
@@ -4284,7 +4383,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>92</v>
       </c>
@@ -4316,7 +4415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>93</v>
       </c>
@@ -4348,7 +4447,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>94</v>
       </c>
@@ -4412,7 +4511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>96</v>
       </c>
@@ -4444,7 +4543,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>97</v>
       </c>
@@ -4476,7 +4575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>98</v>
       </c>
@@ -4508,7 +4607,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>99</v>
       </c>
@@ -4540,7 +4639,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>100</v>
       </c>
@@ -4572,7 +4671,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>101</v>
       </c>
@@ -4604,7 +4703,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>102</v>
       </c>
@@ -4636,7 +4735,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>103</v>
       </c>
@@ -4694,13 +4793,13 @@
         <v>241</v>
       </c>
       <c r="I97" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J97" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>105</v>
       </c>
@@ -4732,7 +4831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>106</v>
       </c>
@@ -4764,7 +4863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>107</v>
       </c>
@@ -4796,7 +4895,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>108</v>
       </c>
@@ -4854,13 +4953,13 @@
         <v>241</v>
       </c>
       <c r="I102" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J102" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>110</v>
       </c>
@@ -4892,7 +4991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>111</v>
       </c>
@@ -4924,7 +5023,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>112</v>
       </c>
@@ -4956,7 +5055,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
         <v>113</v>
       </c>
@@ -4988,7 +5087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
         <v>114</v>
       </c>
@@ -5020,7 +5119,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>115</v>
       </c>
@@ -5052,7 +5151,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
         <v>116</v>
       </c>
@@ -5084,7 +5183,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
         <v>117</v>
       </c>
@@ -5116,7 +5215,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
         <v>118</v>
       </c>
@@ -5148,7 +5247,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
         <v>119</v>
       </c>
@@ -5206,13 +5305,13 @@
         <v>239</v>
       </c>
       <c r="I113" s="2">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="J113" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
         <v>121</v>
       </c>
@@ -5244,7 +5343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
         <v>122</v>
       </c>
@@ -5276,7 +5375,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
         <v>123</v>
       </c>
@@ -5308,7 +5407,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
         <v>124</v>
       </c>
@@ -5340,7 +5439,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
         <v>125</v>
       </c>
@@ -5372,7 +5471,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
         <v>126</v>
       </c>
@@ -5404,7 +5503,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
         <v>127</v>
       </c>
@@ -5436,7 +5535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
         <v>128</v>
       </c>
@@ -5468,7 +5567,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
         <v>129</v>
       </c>
@@ -5500,7 +5599,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
         <v>130</v>
       </c>
@@ -5532,7 +5631,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
         <v>131</v>
       </c>
@@ -5564,7 +5663,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
         <v>132</v>
       </c>
@@ -5596,7 +5695,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
         <v>133</v>
       </c>
@@ -5628,7 +5727,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
         <v>134</v>
       </c>
@@ -5692,7 +5791,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
         <v>136</v>
       </c>
@@ -5724,7 +5823,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
         <v>137</v>
       </c>
@@ -5756,7 +5855,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" s="1" t="s">
         <v>138</v>
       </c>
@@ -5788,7 +5887,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132" s="1" t="s">
         <v>139</v>
       </c>
@@ -5820,7 +5919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133" s="1" t="s">
         <v>140</v>
       </c>
@@ -5852,7 +5951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134" s="1" t="s">
         <v>141</v>
       </c>
@@ -5884,7 +5983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135" s="1" t="s">
         <v>142</v>
       </c>
@@ -5916,7 +6015,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136" s="1" t="s">
         <v>143</v>
       </c>
@@ -5948,7 +6047,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
         <v>144</v>
       </c>
@@ -5980,7 +6079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" s="1" t="s">
         <v>145</v>
       </c>
@@ -6012,7 +6111,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" s="1" t="s">
         <v>146</v>
       </c>
@@ -6044,7 +6143,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140" s="1" t="s">
         <v>147</v>
       </c>
@@ -6076,7 +6175,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" s="1" t="s">
         <v>148</v>
       </c>
@@ -6108,7 +6207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142" s="1" t="s">
         <v>149</v>
       </c>
@@ -6140,7 +6239,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143" s="1" t="s">
         <v>150</v>
       </c>
@@ -6172,7 +6271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144" s="1" t="s">
         <v>151</v>
       </c>
@@ -6204,7 +6303,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145" s="1" t="s">
         <v>152</v>
       </c>
@@ -6236,7 +6335,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
         <v>153</v>
       </c>
@@ -6300,7 +6399,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148" s="1" t="s">
         <v>155</v>
       </c>
@@ -6332,7 +6431,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" s="1" t="s">
         <v>156</v>
       </c>
@@ -6364,7 +6463,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" s="1" t="s">
         <v>157</v>
       </c>
@@ -6396,7 +6495,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151" s="1" t="s">
         <v>158</v>
       </c>
@@ -6428,7 +6527,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" s="1" t="s">
         <v>159</v>
       </c>
@@ -6460,7 +6559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" s="1" t="s">
         <v>372</v>
       </c>
@@ -6492,7 +6591,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" s="1" t="s">
         <v>160</v>
       </c>
@@ -6524,7 +6623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" s="1" t="s">
         <v>161</v>
       </c>
@@ -6556,7 +6655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156" s="1" t="s">
         <v>162</v>
       </c>
@@ -6588,7 +6687,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" s="1" t="s">
         <v>163</v>
       </c>
@@ -6620,7 +6719,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" s="1" t="s">
         <v>164</v>
       </c>
@@ -6652,7 +6751,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159" s="1" t="s">
         <v>165</v>
       </c>
@@ -6684,7 +6783,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160" s="1" t="s">
         <v>166</v>
       </c>
@@ -6716,7 +6815,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161" s="1" t="s">
         <v>167</v>
       </c>
@@ -6748,7 +6847,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A162" s="1" t="s">
         <v>168</v>
       </c>
@@ -6780,7 +6879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A163" s="1" t="s">
         <v>169</v>
       </c>
@@ -6812,7 +6911,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164" s="1" t="s">
         <v>170</v>
       </c>
@@ -6844,7 +6943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A165" s="1" t="s">
         <v>171</v>
       </c>
@@ -6876,7 +6975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166" s="1" t="s">
         <v>172</v>
       </c>
@@ -6934,13 +7033,13 @@
         <v>241</v>
       </c>
       <c r="I167" s="2">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J167" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A168" s="1" t="s">
         <v>174</v>
       </c>
@@ -6972,7 +7071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A169" s="1" t="s">
         <v>175</v>
       </c>
@@ -7004,7 +7103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A170" s="1" t="s">
         <v>176</v>
       </c>
@@ -7036,7 +7135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A171" s="1" t="s">
         <v>177</v>
       </c>
@@ -7068,7 +7167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A172" s="1" t="s">
         <v>178</v>
       </c>
@@ -7100,7 +7199,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A173" s="1" t="s">
         <v>179</v>
       </c>
@@ -7132,7 +7231,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A174" s="1" t="s">
         <v>180</v>
       </c>
@@ -7164,7 +7263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A175" s="1" t="s">
         <v>181</v>
       </c>
@@ -7228,7 +7327,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A177" s="1" t="s">
         <v>183</v>
       </c>
@@ -7260,7 +7359,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A178" s="1" t="s">
         <v>184</v>
       </c>
@@ -7292,7 +7391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A179" s="1" t="s">
         <v>185</v>
       </c>
@@ -7324,7 +7423,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A180" s="1" t="s">
         <v>186</v>
       </c>
@@ -7356,7 +7455,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A181" s="1" t="s">
         <v>187</v>
       </c>
@@ -7388,7 +7487,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A182" s="1" t="s">
         <v>188</v>
       </c>
@@ -7420,7 +7519,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A183" s="1" t="s">
         <v>189</v>
       </c>
@@ -7452,7 +7551,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A184" s="1" t="s">
         <v>190</v>
       </c>
@@ -7484,7 +7583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A185" s="1" t="s">
         <v>191</v>
       </c>
@@ -7516,7 +7615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A186" s="1" t="s">
         <v>192</v>
       </c>
@@ -7548,7 +7647,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A187" s="1" t="s">
         <v>193</v>
       </c>
@@ -7580,7 +7679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A188" s="1" t="s">
         <v>194</v>
       </c>
@@ -7670,13 +7769,13 @@
         <v>241</v>
       </c>
       <c r="I190" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J190" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A191" s="1" t="s">
         <v>197</v>
       </c>
@@ -7708,7 +7807,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A192" s="1" t="s">
         <v>198</v>
       </c>
@@ -7740,7 +7839,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A193" s="1" t="s">
         <v>199</v>
       </c>
@@ -7772,7 +7871,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A194" s="1" t="s">
         <v>200</v>
       </c>
@@ -7804,7 +7903,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A195" s="1" t="s">
         <v>201</v>
       </c>
@@ -7836,7 +7935,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A196" s="1" t="s">
         <v>373</v>
       </c>
@@ -7868,7 +7967,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A197" s="1" t="s">
         <v>202</v>
       </c>
@@ -7900,7 +7999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A198" s="1" t="s">
         <v>203</v>
       </c>
@@ -7932,7 +8031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A199" s="1" t="s">
         <v>204</v>
       </c>
@@ -7964,7 +8063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A200" s="1" t="s">
         <v>205</v>
       </c>
@@ -7996,7 +8095,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A201" s="1" t="s">
         <v>206</v>
       </c>
@@ -8028,7 +8127,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A202" s="1" t="s">
         <v>207</v>
       </c>
@@ -8060,7 +8159,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A203" s="1" t="s">
         <v>208</v>
       </c>
@@ -8092,7 +8191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A204" s="1" t="s">
         <v>209</v>
       </c>
@@ -8182,13 +8281,13 @@
         <v>241</v>
       </c>
       <c r="I206" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J206" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A207" s="1" t="s">
         <v>212</v>
       </c>
@@ -8220,7 +8319,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A208" s="1" t="s">
         <v>213</v>
       </c>
@@ -8252,7 +8351,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A209" s="1" t="s">
         <v>214</v>
       </c>
@@ -8284,7 +8383,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A210" s="1" t="s">
         <v>215</v>
       </c>
@@ -8316,7 +8415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A211" s="1" t="s">
         <v>216</v>
       </c>
@@ -8348,7 +8447,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:10" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A212" s="1" t="s">
         <v>217</v>
       </c>
@@ -8380,7 +8479,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:10" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A213" s="1" t="s">
         <v>218</v>
       </c>
@@ -8412,7 +8511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:10" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A214" s="1" t="s">
         <v>219</v>
       </c>
@@ -8444,7 +8543,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:10" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A215" s="1" t="s">
         <v>220</v>
       </c>
@@ -8476,7 +8575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="216" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:10" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A216" s="1" t="s">
         <v>221</v>
       </c>
@@ -8508,7 +8607,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A217" s="1" t="s">
         <v>222</v>
       </c>
@@ -8540,7 +8639,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A218" s="1" t="s">
         <v>266</v>
       </c>
@@ -8604,7 +8703,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A220" s="1" t="s">
         <v>268</v>
       </c>
@@ -8636,7 +8735,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A221" s="1" t="s">
         <v>269</v>
       </c>
@@ -8668,7 +8767,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A222" s="1" t="s">
         <v>270</v>
       </c>
@@ -8700,7 +8799,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A223" s="1" t="s">
         <v>271</v>
       </c>
@@ -8732,7 +8831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A224" s="1" t="s">
         <v>272</v>
       </c>
@@ -8761,7 +8860,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="225" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A225" s="1" t="s">
         <v>273</v>
       </c>
@@ -8793,7 +8892,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A226" s="1" t="s">
         <v>274</v>
       </c>
@@ -8825,7 +8924,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A227" s="1" t="s">
         <v>275</v>
       </c>
@@ -8857,7 +8956,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A228" s="1" t="s">
         <v>276</v>
       </c>
@@ -8889,7 +8988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A229" s="1" t="s">
         <v>277</v>
       </c>
@@ -8921,7 +9020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="230" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A230" s="1" t="s">
         <v>278</v>
       </c>
@@ -8953,7 +9052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="231" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A231" s="1" t="s">
         <v>279</v>
       </c>
@@ -8985,7 +9084,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="232" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A232" s="1" t="s">
         <v>280</v>
       </c>
@@ -9017,7 +9116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="233" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A233" s="1" t="s">
         <v>281</v>
       </c>
@@ -9049,7 +9148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="234" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A234" s="1" t="s">
         <v>282</v>
       </c>
@@ -9081,7 +9180,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="235" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A235" s="1" t="s">
         <v>283</v>
       </c>
@@ -9113,7 +9212,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="236" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A236" s="1" t="s">
         <v>284</v>
       </c>
@@ -9145,7 +9244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="237" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A237" s="1" t="s">
         <v>285</v>
       </c>
@@ -9177,7 +9276,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="238" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A238" s="1" t="s">
         <v>286</v>
       </c>
@@ -9209,7 +9308,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="239" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A239" s="1" t="s">
         <v>287</v>
       </c>
@@ -9241,7 +9340,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="240" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A240" s="1" t="s">
         <v>288</v>
       </c>
@@ -9273,7 +9372,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="241" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A241" s="1" t="s">
         <v>289</v>
       </c>
@@ -9305,7 +9404,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="242" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A242" s="1" t="s">
         <v>290</v>
       </c>
@@ -9337,7 +9436,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="243" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A243" s="1" t="s">
         <v>291</v>
       </c>
@@ -9369,7 +9468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="244" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A244" s="1" t="s">
         <v>292</v>
       </c>
@@ -9401,7 +9500,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="245" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A245" s="1" t="s">
         <v>293</v>
       </c>
@@ -9433,7 +9532,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="246" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A246" s="1" t="s">
         <v>294</v>
       </c>
@@ -9465,7 +9564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="247" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A247" s="1" t="s">
         <v>295</v>
       </c>
@@ -9497,7 +9596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="248" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A248" s="1" t="s">
         <v>296</v>
       </c>
@@ -9529,7 +9628,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="249" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A249" s="1" t="s">
         <v>297</v>
       </c>
@@ -9561,7 +9660,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="250" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A250" s="1" t="s">
         <v>298</v>
       </c>
@@ -9593,7 +9692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="251" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A251" s="1" t="s">
         <v>299</v>
       </c>
@@ -9625,7 +9724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="252" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A252" s="1" t="s">
         <v>300</v>
       </c>
@@ -9657,7 +9756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="253" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A253" s="1" t="s">
         <v>301</v>
       </c>
@@ -9689,7 +9788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="254" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A254" s="1" t="s">
         <v>302</v>
       </c>
@@ -9721,7 +9820,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="255" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A255" s="1" t="s">
         <v>303</v>
       </c>
@@ -9753,7 +9852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="256" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A256" s="1" t="s">
         <v>304</v>
       </c>
@@ -9785,7 +9884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="257" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A257" s="1" t="s">
         <v>305</v>
       </c>
@@ -9817,7 +9916,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="258" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A258" s="1" t="s">
         <v>306</v>
       </c>
@@ -9849,7 +9948,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="259" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A259" s="1" t="s">
         <v>307</v>
       </c>
@@ -9881,7 +9980,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="260" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A260" s="1" t="s">
         <v>308</v>
       </c>
@@ -9913,7 +10012,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="261" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A261" s="1" t="s">
         <v>309</v>
       </c>
@@ -9945,7 +10044,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="262" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A262" s="1" t="s">
         <v>310</v>
       </c>
@@ -9977,7 +10076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="263" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A263" s="1" t="s">
         <v>311</v>
       </c>
@@ -10009,7 +10108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="264" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A264" s="1" t="s">
         <v>312</v>
       </c>
@@ -10041,7 +10140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="265" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A265" s="1" t="s">
         <v>313</v>
       </c>
@@ -10073,7 +10172,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="266" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A266" s="1" t="s">
         <v>314</v>
       </c>
@@ -10105,7 +10204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="267" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A267" s="1" t="s">
         <v>315</v>
       </c>
@@ -10137,7 +10236,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="268" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A268" s="1" t="s">
         <v>316</v>
       </c>
@@ -10169,7 +10268,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="269" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A269" s="1" t="s">
         <v>317</v>
       </c>
@@ -10201,7 +10300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="270" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A270" s="1" t="s">
         <v>318</v>
       </c>
@@ -10233,7 +10332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="271" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A271" s="1" t="s">
         <v>319</v>
       </c>
@@ -10265,7 +10364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="272" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A272" s="1" t="s">
         <v>320</v>
       </c>
@@ -10297,7 +10396,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="273" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A273" s="1" t="s">
         <v>321</v>
       </c>
@@ -10329,7 +10428,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="274" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A274" s="1" t="s">
         <v>322</v>
       </c>
@@ -10361,7 +10460,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="275" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A275" s="1" t="s">
         <v>323</v>
       </c>
@@ -10393,7 +10492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="276" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A276" s="1" t="s">
         <v>324</v>
       </c>
@@ -10425,7 +10524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="277" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A277" s="1" t="s">
         <v>325</v>
       </c>
@@ -10457,7 +10556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="278" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A278" s="1" t="s">
         <v>326</v>
       </c>
@@ -10489,7 +10588,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="279" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A279" s="1" t="s">
         <v>327</v>
       </c>
@@ -10521,7 +10620,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="280" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A280" s="1" t="s">
         <v>328</v>
       </c>
@@ -10553,7 +10652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="281" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A281" s="1" t="s">
         <v>329</v>
       </c>
@@ -10585,7 +10684,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="282" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A282" s="1" t="s">
         <v>330</v>
       </c>
@@ -10617,7 +10716,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="283" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A283" s="1" t="s">
         <v>331</v>
       </c>
@@ -10649,7 +10748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="284" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A284" s="1" t="s">
         <v>332</v>
       </c>
@@ -10681,7 +10780,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="285" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A285" s="1" t="s">
         <v>333</v>
       </c>
@@ -10713,7 +10812,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="286" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A286" s="1" t="s">
         <v>334</v>
       </c>
@@ -10745,7 +10844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="287" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A287" s="1" t="s">
         <v>335</v>
       </c>
@@ -10777,7 +10876,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="288" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A288" s="1" t="s">
         <v>336</v>
       </c>
@@ -10809,7 +10908,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="289" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A289" s="1" t="s">
         <v>337</v>
       </c>
@@ -10841,7 +10940,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="290" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A290" s="1" t="s">
         <v>338</v>
       </c>
@@ -10873,7 +10972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="291" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A291" s="1" t="s">
         <v>339</v>
       </c>
@@ -10905,7 +11004,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="292" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A292" s="1" t="s">
         <v>340</v>
       </c>
@@ -10937,7 +11036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="293" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A293" s="1" t="s">
         <v>341</v>
       </c>
@@ -10969,7 +11068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="294" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A294" s="1" t="s">
         <v>342</v>
       </c>
@@ -11001,7 +11100,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="295" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A295" s="1" t="s">
         <v>343</v>
       </c>
@@ -11033,7 +11132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="296" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A296" s="1" t="s">
         <v>344</v>
       </c>
@@ -11065,7 +11164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="297" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A297" s="1" t="s">
         <v>345</v>
       </c>
@@ -11097,7 +11196,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="298" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A298" s="1" t="s">
         <v>346</v>
       </c>
@@ -11129,7 +11228,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="299" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A299" s="1" t="s">
         <v>347</v>
       </c>
@@ -11161,7 +11260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="300" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A300" s="1" t="s">
         <v>348</v>
       </c>
@@ -11193,7 +11292,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="301" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A301" s="1" t="s">
         <v>349</v>
       </c>
@@ -11225,7 +11324,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="302" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A302" s="1" t="s">
         <v>350</v>
       </c>
@@ -11257,7 +11356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="303" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A303" s="1" t="s">
         <v>351</v>
       </c>
@@ -11289,7 +11388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="304" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A304" s="1" t="s">
         <v>352</v>
       </c>
@@ -11321,7 +11420,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="305" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A305" s="1" t="s">
         <v>353</v>
       </c>
@@ -11353,7 +11452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="306" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A306" s="1" t="s">
         <v>354</v>
       </c>
@@ -11385,7 +11484,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="307" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A307" s="1" t="s">
         <v>355</v>
       </c>
@@ -11417,7 +11516,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="308" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A308" s="1" t="s">
         <v>356</v>
       </c>
@@ -11449,7 +11548,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="309" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A309" s="1" t="s">
         <v>357</v>
       </c>
@@ -11481,7 +11580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="310" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A310" s="1" t="s">
         <v>358</v>
       </c>
@@ -11513,7 +11612,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="311" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A311" s="1" t="s">
         <v>359</v>
       </c>
@@ -11545,7 +11644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="312" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A312" s="1" t="s">
         <v>360</v>
       </c>
@@ -11577,7 +11676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="313" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A313" s="1" t="s">
         <v>374</v>
       </c>
@@ -11609,7 +11708,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="314" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A314" s="1" t="s">
         <v>375</v>
       </c>
@@ -11641,7 +11740,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="315" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A315" s="1" t="s">
         <v>376</v>
       </c>
@@ -11673,7 +11772,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="316" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A316" s="1" t="s">
         <v>377</v>
       </c>
@@ -11705,7 +11804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="317" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A317" s="1" t="s">
         <v>378</v>
       </c>
@@ -11737,7 +11836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="318" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A318" s="1" t="s">
         <v>379</v>
       </c>
@@ -11769,7 +11868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="319" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A319" s="1" t="s">
         <v>380</v>
       </c>
@@ -11801,7 +11900,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="320" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A320" s="1" t="s">
         <v>381</v>
       </c>
@@ -11833,7 +11932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="321" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A321" s="1" t="s">
         <v>382</v>
       </c>
@@ -11865,7 +11964,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="322" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A322" s="1" t="s">
         <v>383</v>
       </c>
@@ -11897,7 +11996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="323" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A323" s="1" t="s">
         <v>384</v>
       </c>
@@ -11929,7 +12028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="324" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A324" s="1" t="s">
         <v>388</v>
       </c>
@@ -11961,7 +12060,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="325" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A325" s="1" t="s">
         <v>389</v>
       </c>
@@ -11993,7 +12092,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="326" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A326" s="1" t="s">
         <v>390</v>
       </c>
@@ -12025,7 +12124,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="327" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A327" s="1" t="s">
         <v>391</v>
       </c>
@@ -12057,7 +12156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="328" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A328" s="1" t="s">
         <v>392</v>
       </c>
@@ -12090,8 +12189,16 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:J328" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="4">
+      <filters>
+        <filter val="Nuevo CAS"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update data +  config
</commit_message>
<xml_diff>
--- a/data/metas.xlsx
+++ b/data/metas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROYECTOS - 2026 (DEV)\DEV - POI\Insights_POI\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{373B7A82-B8CF-4BED-A9E8-77BB864CE793}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E14D1941-D431-4A22-949D-63ED74C069F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1287,14 +1287,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1500,19 +1498,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A94C55CA-EA62-4689-9D49-11D174A7C6C9}" name="Tabla1" displayName="Tabla1" ref="C1:J328" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A94C55CA-EA62-4689-9D49-11D174A7C6C9}" name="Tabla1" displayName="Tabla1" ref="C1:J328" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
   <autoFilter ref="C1:J328" xr:uid="{A94C55CA-EA62-4689-9D49-11D174A7C6C9}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{762B2E27-3995-4311-9C01-127F54E0F93A}" name="MES" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{1456C7DD-C371-4A0D-84AA-97597FFDA208}" name="PROGRAMA" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{811B7471-2536-48E0-893B-9FF46C5EB5D8}" name="ESPECIALISTA" dataDxfId="7">
+    <tableColumn id="1" xr3:uid="{762B2E27-3995-4311-9C01-127F54E0F93A}" name="MES" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{1456C7DD-C371-4A0D-84AA-97597FFDA208}" name="PROGRAMA" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{811B7471-2536-48E0-893B-9FF46C5EB5D8}" name="ESPECIALISTA" dataDxfId="5">
       <calculatedColumnFormula>+UPPER(Tabla1[[#This Row],[ESPECIALISTA]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{A3321876-A637-4BB9-BCA9-0B61CA20762C}" name="TIPO_SERVICIO" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{17E9C769-C3BE-41B6-A041-FD066E817C9D}" name="COMPLEJIDAD" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{6F1113B5-3201-4922-BF51-C879991BF4FC}" name="TIPO_TAREA" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{30CFDF01-E2A1-4489-87A3-FA3F0F99C05D}" name="META_CANTIDAD" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{56019005-51AF-4C82-90C1-96AC0FF918B6}" name="META_FOCALIZADOS" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{A3321876-A637-4BB9-BCA9-0B61CA20762C}" name="TIPO_SERVICIO" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{17E9C769-C3BE-41B6-A041-FD066E817C9D}" name="COMPLEJIDAD" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{6F1113B5-3201-4922-BF51-C879991BF4FC}" name="TIPO_TAREA" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{30CFDF01-E2A1-4489-87A3-FA3F0F99C05D}" name="META_CANTIDAD" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{56019005-51AF-4C82-90C1-96AC0FF918B6}" name="META_FOCALIZADOS" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1901,7 +1899,7 @@
       <c r="H2" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="I2" s="5">
+      <c r="I2" s="1">
         <v>17</v>
       </c>
       <c r="J2" s="1">
@@ -1934,7 +1932,7 @@
       <c r="H3" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="I3" s="5">
+      <c r="I3" s="1">
         <v>6</v>
       </c>
       <c r="J3" s="1">
@@ -1967,7 +1965,7 @@
       <c r="H4" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="I4" s="6">
+      <c r="I4" s="2">
         <v>17</v>
       </c>
       <c r="J4" s="1">
@@ -2000,7 +1998,7 @@
       <c r="H5" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="I5" s="5">
+      <c r="I5" s="1">
         <v>20</v>
       </c>
       <c r="J5" s="1">
@@ -2033,7 +2031,7 @@
       <c r="H6" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="I6" s="6">
+      <c r="I6" s="2">
         <v>15</v>
       </c>
       <c r="J6" s="1">
@@ -2066,7 +2064,7 @@
       <c r="H7" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="I7" s="5">
+      <c r="I7" s="1">
         <v>1</v>
       </c>
       <c r="J7" s="1">
@@ -2099,7 +2097,7 @@
       <c r="H8" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="I8" s="5">
+      <c r="I8" s="1">
         <v>75</v>
       </c>
       <c r="J8" s="1">
@@ -2132,7 +2130,7 @@
       <c r="H9" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="I9" s="6">
+      <c r="I9" s="2">
         <v>16</v>
       </c>
       <c r="J9" s="1">
@@ -2165,7 +2163,7 @@
       <c r="H10" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="I10" s="5">
+      <c r="I10" s="1">
         <v>5</v>
       </c>
       <c r="J10" s="1">
@@ -2198,7 +2196,7 @@
       <c r="H11" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="I11" s="5">
+      <c r="I11" s="1">
         <v>15</v>
       </c>
       <c r="J11" s="1">

</xml_diff>